<commit_message>
Upload GitHub Summary - 2026-04-10 04:12:07
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>April 9, 2026</t>
+    <t>April 10, 2026</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-04-11 03:41:28
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>April 10, 2026</t>
+    <t>April 11, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3143</v>
+        <v>3144</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-04-15 04:12:13
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>April 14, 2026</t>
+    <t>April 15, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3144</v>
+        <v>3145</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-04-22 04:11:53
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>April 21, 2026</t>
+    <t>April 22, 2026</t>
   </si>
 </sst>
 </file>
@@ -689,7 +689,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -707,7 +707,7 @@
         <v>12</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -948,7 +948,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -966,7 +966,7 @@
         <v>48</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-04-24 04:21:28
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>April 23, 2026</t>
+    <t>April 24, 2026</t>
   </si>
 </sst>
 </file>
@@ -497,7 +497,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -515,7 +515,7 @@
         <v>46</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3145</v>
+        <v>3146</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-04-25 03:55:30
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>April 24, 2026</t>
+    <t>April 25, 2026</t>
   </si>
 </sst>
 </file>
@@ -658,7 +658,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C9">
         <v>20</v>
@@ -676,7 +676,7 @@
         <v>4</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3146</v>
+        <v>3147</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -917,7 +917,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C9">
         <v>54</v>
@@ -935,7 +935,7 @@
         <v>4</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-05-01 04:53:57
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>April 30, 2026</t>
+    <t>May 1, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3147</v>
+        <v>3148</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-05-08 04:19:47
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>May 7, 2026</t>
+    <t>May 8, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3148</v>
+        <v>3149</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-05-10 04:50:18
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>May 9, 2026</t>
+    <t>May 10, 2026</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-05-15 04:57:00
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>May 14, 2026</t>
+    <t>May 15, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3149</v>
+        <v>3151</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-05-16 04:33:41
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>May 15, 2026</t>
+    <t>May 16, 2026</t>
   </si>
 </sst>
 </file>
@@ -497,7 +497,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -515,7 +515,7 @@
         <v>46</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3151</v>
+        <v>3152</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-05-19 05:08:12
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>May 18, 2026</t>
+    <t>May 19, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3152</v>
+        <v>3155</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-05-27 05:23:32
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>May 26, 2026</t>
+    <t>May 27, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3155</v>
+        <v>3158</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-05-28 05:15:54
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>May 27, 2026</t>
+    <t>May 28, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3158</v>
+        <v>3168</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>113</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-05-29 05:18:55
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>May 28, 2026</t>
+    <t>May 29, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3168</v>
+        <v>3170</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-06-03 06:10:03
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 2, 2026</t>
+    <t>June 3, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3170</v>
+        <v>3171</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-06-05 05:25:17
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 4, 2026</t>
+    <t>June 5, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3171</v>
+        <v>3173</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-06-06 05:00:18
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 5, 2026</t>
+    <t>June 6, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3173</v>
+        <v>3174</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-06-10 05:25:09
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 9, 2026</t>
+    <t>June 10, 2026</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-06-11 05:59:32
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 10, 2026</t>
+    <t>June 11, 2026</t>
   </si>
 </sst>
 </file>
@@ -658,25 +658,25 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="C9">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D9">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E9">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="F9">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -917,25 +917,25 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>133</v>
+        <v>26</v>
       </c>
       <c r="C9">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="D9">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E9">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="F9">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-06-12 05:55:17
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 11, 2026</t>
+    <t>June 12, 2026</t>
   </si>
 </sst>
 </file>
@@ -658,25 +658,25 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="C9">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -917,25 +917,25 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>26</v>
+        <v>133</v>
       </c>
       <c r="C9">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="D9">
+        <v>21</v>
+      </c>
+      <c r="E9">
+        <v>27</v>
+      </c>
+      <c r="F9">
+        <v>17</v>
+      </c>
+      <c r="G9">
+        <v>4</v>
+      </c>
+      <c r="H9">
         <v>2</v>
-      </c>
-      <c r="E9">
-        <v>4</v>
-      </c>
-      <c r="F9">
-        <v>2</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-      <c r="H9">
-        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-06-13 05:25:41
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 12, 2026</t>
+    <t>June 13, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3174</v>
+        <v>3176</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-06-19 06:26:25
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 18, 2026</t>
+    <t>June 19, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3176</v>
+        <v>3177</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-06-24 05:11:00
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 23, 2026</t>
+    <t>June 24, 2026</t>
   </si>
 </sst>
 </file>
@@ -689,7 +689,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -707,7 +707,7 @@
         <v>12</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -948,7 +948,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -966,7 +966,7 @@
         <v>48</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-06-30 05:12:41
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 29, 2026</t>
+    <t>June 30, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3177</v>
+        <v>3178</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-07-01 05:47:38
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>June 30, 2026</t>
+    <t>July 1, 2026</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-07-03 01:41:28
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>July 2, 2026</t>
+    <t>July 3, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3178</v>
+        <v>3184</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-07-08 01:41:28
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>July 7, 2026</t>
+    <t>July 8, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3184</v>
+        <v>3187</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-07-10 01:42:32
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>July 9, 2026</t>
+    <t>July 10, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3187</v>
+        <v>3188</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-07-11 01:40:42
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>July 10, 2026</t>
+    <t>July 11, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3188</v>
+        <v>3189</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-07-21 01:41:54
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>July 20, 2026</t>
+    <t>July 21, 2026</t>
   </si>
 </sst>
 </file>
@@ -497,7 +497,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="C2">
         <v>130</v>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-07-22 01:41:28
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>July 21, 2026</t>
+    <t>July 22, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3189</v>
+        <v>3191</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-07-24 14:16:43
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3191</v>
+        <v>3192</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-07-30 01:40:21
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>July 29, 2026</t>
+    <t>July 30, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3192</v>
+        <v>3193</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-01 01:41:44
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>July 31, 2026</t>
+    <t>August 1, 2026</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-10 01:37:11
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 9, 2026</t>
+    <t>August 10, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3193</v>
+        <v>3199</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-12 01:37:22
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 11, 2026</t>
+    <t>August 12, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3199</v>
+        <v>3200</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-14 01:37:15
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 13, 2026</t>
+    <t>August 14, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3200</v>
+        <v>3201</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-15 01:34:05
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 14, 2026</t>
+    <t>August 15, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3201</v>
+        <v>3202</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-18 01:34:01
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 17, 2026</t>
+    <t>August 18, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3202</v>
+        <v>3207</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-19 01:34:17
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 18, 2026</t>
+    <t>August 19, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3207</v>
+        <v>3212</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-20 01:34:02
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 19, 2026</t>
+    <t>August 20, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3212</v>
+        <v>3215</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-25 01:34:12
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 24, 2026</t>
+    <t>August 25, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3215</v>
+        <v>3216</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-26 01:34:39
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 25, 2026</t>
+    <t>August 26, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3216</v>
+        <v>3217</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-28 03:51:09
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 27, 2026</t>
+    <t>August 28, 2026</t>
   </si>
 </sst>
 </file>
@@ -689,7 +689,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -704,10 +704,10 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3217</v>
+        <v>3219</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -948,7 +948,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -963,10 +963,10 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="H11">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-08-29 01:18:27
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 28, 2026</t>
+    <t>August 29, 2026</t>
   </si>
 </sst>
 </file>
@@ -549,7 +549,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -567,7 +567,7 @@
         <v>2</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -689,7 +689,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -704,10 +704,10 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3219</v>
+        <v>3222</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -808,7 +808,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -826,7 +826,7 @@
         <v>4</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -948,7 +948,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -963,10 +963,10 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-01 01:36:54
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>August 31, 2026</t>
+    <t>September 1, 2026</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-03 01:34:55
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 2, 2026</t>
+    <t>September 3, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3222</v>
+        <v>3226</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-04 01:25:31
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 3, 2026</t>
+    <t>September 4, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3226</v>
+        <v>3227</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-06 01:30:24
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 5, 2026</t>
+    <t>September 6, 2026</t>
   </si>
 </sst>
 </file>
@@ -497,7 +497,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -515,7 +515,7 @@
         <v>46</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3227</v>
+        <v>3228</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-09 01:30:16
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 8, 2026</t>
+    <t>September 9, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3228</v>
+        <v>3229</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-10 01:27:20
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 9, 2026</t>
+    <t>September 10, 2026</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>